<commit_message>
Suite as on: 4th October
</commit_message>
<xml_diff>
--- a/testData/DDT_testdata.xlsx
+++ b/testData/DDT_testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bba80875e260e8e3/Desktop/OrangeHRM_Test_Suite/testData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="246" documentId="8_{F5AB6998-FAF7-4A82-A8FC-A21EFAED1A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DB76534-1AEF-41B6-AE85-613A8D6E941E}"/>
+  <xr:revisionPtr revIDLastSave="287" documentId="8_{F5AB6998-FAF7-4A82-A8FC-A21EFAED1A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D226D60-951D-41C8-B358-CC8F611DD434}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{4CB12ADF-4430-4E69-A35C-A24127896C07}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="118">
   <si>
     <t>File Path</t>
   </si>
@@ -327,13 +327,70 @@
     <t>Schedule Interview and Reject</t>
   </si>
   <si>
-    <t xml:space="preserve">Offer Accept and </t>
-  </si>
-  <si>
     <t>Interview pass/fail/reject</t>
   </si>
   <si>
     <t>Payroll Administrator</t>
+  </si>
+  <si>
+    <t>Kelly</t>
+  </si>
+  <si>
+    <t>Erin</t>
+  </si>
+  <si>
+    <t>Hannon</t>
+  </si>
+  <si>
+    <t>kelly@dundermifflin.com</t>
+  </si>
+  <si>
+    <t>Current Receptionist</t>
+  </si>
+  <si>
+    <t>Angella</t>
+  </si>
+  <si>
+    <t>Noelle</t>
+  </si>
+  <si>
+    <t>Martin</t>
+  </si>
+  <si>
+    <t>angella@dundermifflin.com</t>
+  </si>
+  <si>
+    <t>Second Round of Interview</t>
+  </si>
+  <si>
+    <t>Bailey</t>
+  </si>
+  <si>
+    <t>Howard</t>
+  </si>
+  <si>
+    <t>Digitization expert</t>
+  </si>
+  <si>
+    <t>ryan@dunddermifflin.com</t>
+  </si>
+  <si>
+    <t>Ryan</t>
+  </si>
+  <si>
+    <t>Gabriel</t>
+  </si>
+  <si>
+    <t>Susan</t>
+  </si>
+  <si>
+    <t>Lewis</t>
+  </si>
+  <si>
+    <t>lewis@dundermifflin.com</t>
+  </si>
+  <si>
+    <t>Hired</t>
   </si>
 </sst>
 </file>
@@ -1020,7 +1077,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B4EA1A-0C17-449A-9C5C-7637EE779B83}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" customWidth="1"/>
@@ -1081,7 +1138,7 @@
         <v>77</v>
       </c>
       <c r="E2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F2">
         <v>8786564</v>
@@ -1113,7 +1170,7 @@
         <v>75</v>
       </c>
       <c r="E3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F3">
         <v>7987643</v>
@@ -1145,7 +1202,7 @@
         <v>76</v>
       </c>
       <c r="E4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F4">
         <v>9086954</v>
@@ -1177,7 +1234,7 @@
         <v>84</v>
       </c>
       <c r="E5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F5">
         <v>9090294</v>
@@ -1189,7 +1246,7 @@
         <v>85</v>
       </c>
       <c r="I5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J5" t="s">
         <v>86</v>
@@ -1209,7 +1266,7 @@
         <v>90</v>
       </c>
       <c r="E6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F6">
         <v>9088765</v>
@@ -1221,10 +1278,135 @@
         <v>64</v>
       </c>
       <c r="I6" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="J6" t="s">
         <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E7" t="s">
+        <v>97</v>
+      </c>
+      <c r="F7">
+        <v>1223545</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>64</v>
+      </c>
+      <c r="I7" t="s">
+        <v>107</v>
+      </c>
+      <c r="J7" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C8" t="s">
+        <v>105</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E8" t="s">
+        <v>97</v>
+      </c>
+      <c r="F8">
+        <v>9567855</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" t="s">
+        <v>63</v>
+      </c>
+      <c r="I8" t="s">
+        <v>93</v>
+      </c>
+      <c r="J8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" t="s">
+        <v>109</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E9" t="s">
+        <v>97</v>
+      </c>
+      <c r="F9">
+        <v>2367855</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9" t="s">
+        <v>85</v>
+      </c>
+      <c r="J9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B10" t="s">
+        <v>114</v>
+      </c>
+      <c r="C10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="E10" t="s">
+        <v>97</v>
+      </c>
+      <c r="F10">
+        <v>7337955</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I10" t="s">
+        <v>117</v>
+      </c>
+      <c r="J10" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1234,6 +1416,10 @@
     <hyperlink ref="D4" r:id="rId3" xr:uid="{17EF0CF1-022E-48E5-9738-BC62C519B7E9}"/>
     <hyperlink ref="D5" r:id="rId4" xr:uid="{99619FBD-99BE-481A-BB70-79ECF82AE1D6}"/>
     <hyperlink ref="D6" r:id="rId5" xr:uid="{5E01DD81-9C36-4E2C-83A9-25C2BE2F9BEF}"/>
+    <hyperlink ref="D7" r:id="rId6" xr:uid="{079FF018-7EA3-4A84-B92A-3085145A6ED2}"/>
+    <hyperlink ref="D8" r:id="rId7" xr:uid="{B9FA7CB8-867D-4293-BD0A-C8EE2693F854}"/>
+    <hyperlink ref="D9" r:id="rId8" xr:uid="{A03A9FAC-3976-402D-9C93-052D78B3F37B}"/>
+    <hyperlink ref="D10" r:id="rId9" xr:uid="{21DDBB41-3181-44BA-939D-5C78F237A4A6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>